<commit_message>
test: Cập nhật kịch bản kiểm thử API (chuẩn bị trước khi BE hoàn thiện REST API)
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -1,17 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
+  <bookViews>
+    <workbookView windowWidth="22188" windowHeight="9000" activeTab="1"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Bảng Kịch Bản Kiểm Thử Hoàn Chỉ" sheetId="1" r:id="rId5"/>
+    <sheet name="Bảng Kịch Bản Kiểm Thử Hoàn Chỉ" sheetId="1" r:id="rId1"/>
+    <sheet name="API Test Cases" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="178">
   <si>
     <t>Mã TC</t>
   </si>
@@ -449,90 +466,996 @@
   </si>
   <si>
     <t>Hệ thống chặn và báo lỗi: "Không thể xóa chi nhánh đang hoạt động. Vui lòng vô hiệu hóa".</t>
+  </si>
+  <si>
+    <t>Test Case ID</t>
+  </si>
+  <si>
+    <t>Module</t>
+  </si>
+  <si>
+    <t>Phương thức</t>
+  </si>
+  <si>
+    <t>API Endpoint (Dự kiến)</t>
+  </si>
+  <si>
+    <t>Dữ liệu đầu vào (Request Body)</t>
+  </si>
+  <si>
+    <t>Kết quả mong đợi (Expected Output)</t>
+  </si>
+  <si>
+    <t>Trạng thái (Status)</t>
+  </si>
+  <si>
+    <t>API-TC-01</t>
+  </si>
+  <si>
+    <t>Auth</t>
+  </si>
+  <si>
+    <t>POST</t>
+  </si>
+  <si>
+    <t>/api/auth/login</t>
+  </si>
+  <si>
+    <t>{ "email": "admin@gym.com", "password": "123" }</t>
+  </si>
+  <si>
+    <t>Trả về Status 200 OK. Kèm Token đăng nhập.</t>
+  </si>
+  <si>
+    <t>Untested (Blocked)</t>
+  </si>
+  <si>
+    <t>API-TC-02</t>
+  </si>
+  <si>
+    <t>{ "email": "admin@gym.com", "password": "sai" }</t>
+  </si>
+  <si>
+    <t>Trả về Status 401 Unauthorized. Báo lỗi sai pass.</t>
+  </si>
+  <si>
+    <t>API-TC-03</t>
+  </si>
+  <si>
+    <t>Packages</t>
+  </si>
+  <si>
+    <t>GET</t>
+  </si>
+  <si>
+    <t>/api/packages</t>
+  </si>
+  <si>
+    <t>(Không có)</t>
+  </si>
+  <si>
+    <t>Trả về Status 200 OK. Dữ liệu mảng JSON chứa đúng 5 gói tập.</t>
+  </si>
+  <si>
+    <t>API-TC-04</t>
+  </si>
+  <si>
+    <t>Classes</t>
+  </si>
+  <si>
+    <t>/api/classes</t>
+  </si>
+  <si>
+    <t>Trả về Status 200 OK. Dữ liệu mảng JSON chứa danh sách các lớp học.</t>
+  </si>
+  <si>
+    <t>API-TC-05</t>
+  </si>
+  <si>
+    <t>Booking</t>
+  </si>
+  <si>
+    <t>/api/classes/book</t>
+  </si>
+  <si>
+    <t>{ "class_id": 1, "member_id": 2 }</t>
+  </si>
+  <si>
+    <t>Trả về Status 200 OK. Thông báo đặt lớp thành công.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
-    <font>
-      <sz val="10.0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="26">
+    <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF444746"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
-  <borders count="1">
-    <border/>
+  <borders count="10">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1F1F1F"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1F1F1F"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF1F1F1F"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1F1F1F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+  <cellXfs count="7">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+  <cellStyles count="49">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="13">
     <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-      <border/>
+      <font>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
     </dxf>
     <dxf>
-      <font/>
+      <font>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF356854"/>
           <bgColor rgb="FF356854"/>
         </patternFill>
       </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF6F8F9"/>
-          <bgColor rgb="FFF6F8F9"/>
-        </patternFill>
-      </fill>
-      <border/>
     </dxf>
     <dxf>
       <border>
@@ -552,43 +1475,40 @@
     </dxf>
   </dxfs>
   <tableStyles count="1">
-    <tableStyle count="4" pivot="0" name="Bảng Kịch Bản Kiểm Thử Hoàn Chỉ-style">
-      <tableStyleElement dxfId="1" type="headerRow"/>
-      <tableStyleElement dxfId="2" type="firstRowStripe"/>
-      <tableStyleElement dxfId="3" type="secondRowStripe"/>
-      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    <tableStyle name="Bảng Kịch Bản Kiểm Thử Hoàn Chỉ-style" pivot="0" count="4" xr9:uid="{30E614A9-3B57-43FD-B4DF-F723546CBBD8}">
+      <tableStyleElement type="wholeTable" dxfId="12"/>
+      <tableStyleElement type="headerRow" dxfId="11"/>
+      <tableStyleElement type="firstRowStripe" dxfId="10"/>
+      <tableStyleElement type="secondRowStripe" dxfId="9"/>
     </tableStyle>
   </tableStyles>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:I21" displayName="Bảng_1" name="Bảng_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bảng_1" displayName="Bảng_1" ref="A1:I21">
   <tableColumns count="9">
-    <tableColumn name="Mã TC" id="1"/>
-    <tableColumn name="Mã UC Tham chiếu" id="2"/>
-    <tableColumn name="Module / Chức năng" id="3"/>
-    <tableColumn name="Tên Kịch Bản (Test Case Name)" id="4"/>
-    <tableColumn name="Tiền điều kiện (Precondition)" id="5"/>
-    <tableColumn name="Các bước thực hiện (Steps)" id="6"/>
-    <tableColumn name="Dữ liệu đầu vào (Input Data)" id="7"/>
-    <tableColumn name="Kết quả mong đợi (Expected Result)" id="8"/>
-    <tableColumn name="Phân loại" id="9"/>
+    <tableColumn id="1" name="Mã TC" dataDxfId="0"/>
+    <tableColumn id="2" name="Mã UC Tham chiếu" dataDxfId="1"/>
+    <tableColumn id="3" name="Module / Chức năng" dataDxfId="2"/>
+    <tableColumn id="4" name="Tên Kịch Bản (Test Case Name)" dataDxfId="3"/>
+    <tableColumn id="5" name="Tiền điều kiện (Precondition)" dataDxfId="4"/>
+    <tableColumn id="6" name="Các bước thực hiện (Steps)" dataDxfId="5"/>
+    <tableColumn id="7" name="Dữ liệu đầu vào (Input Data)" dataDxfId="6"/>
+    <tableColumn id="8" name="Kết quả mong đợi (Expected Result)" dataDxfId="7"/>
+    <tableColumn id="9" name="Phân loại" dataDxfId="8"/>
   </tableColumns>
-  <tableStyleInfo name="Bảng Kịch Bản Kiểm Thử Hoàn Chỉ-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="Bảng Kịch Bản Kiểm Thử Hoàn Chỉ-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -778,635 +1698,791 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:I21"/>
+  <sheetFormatPr defaultColWidth="12.6296296296296" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="19.5"/>
-    <col customWidth="1" min="3" max="3" width="30.5"/>
-    <col customWidth="1" min="4" max="8" width="37.63"/>
-    <col customWidth="1" min="9" max="9" width="22.0"/>
+    <col min="2" max="2" width="19.5" customWidth="1"/>
+    <col min="3" max="3" width="30.5" customWidth="1"/>
+    <col min="4" max="8" width="37.6296296296296" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="22.5" customHeight="1" spans="1:9">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" ht="22.5" customHeight="1">
-      <c r="A2" s="2" t="s">
+    <row r="2" ht="22.5" customHeight="1" spans="1:9">
+      <c r="A2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="2" t="s">
+    <row r="3" ht="22.5" customHeight="1" spans="1:9">
+      <c r="A3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="6" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="2" t="s">
+    <row r="4" ht="22.5" customHeight="1" spans="1:9">
+      <c r="A4" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="2" t="s">
+    <row r="5" ht="22.5" customHeight="1" spans="1:9">
+      <c r="A5" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="I5" s="6" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="2" t="s">
+    <row r="6" ht="22.5" customHeight="1" spans="1:9">
+      <c r="A6" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="G6" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="I6" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="2" t="s">
+    <row r="7" ht="22.5" customHeight="1" spans="1:9">
+      <c r="A7" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="I7" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="2" t="s">
+    <row r="8" ht="22.5" customHeight="1" spans="1:9">
+      <c r="A8" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="I8" s="6" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="2" t="s">
+    <row r="9" ht="22.5" customHeight="1" spans="1:9">
+      <c r="A9" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G9" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="I9" s="6" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="10" ht="22.5" customHeight="1">
-      <c r="A10" s="2" t="s">
+    <row r="10" ht="22.5" customHeight="1" spans="1:9">
+      <c r="A10" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I10" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="11" ht="22.5" customHeight="1">
-      <c r="A11" s="2" t="s">
+    <row r="11" ht="22.5" customHeight="1" spans="1:9">
+      <c r="A11" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="G11" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="I11" s="6" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="12" ht="22.5" customHeight="1">
-      <c r="A12" s="2" t="s">
+    <row r="12" ht="22.5" customHeight="1" spans="1:9">
+      <c r="A12" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="G12" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="H12" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="I12" s="2" t="s">
+      <c r="I12" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="13" ht="22.5" customHeight="1">
-      <c r="A13" s="2" t="s">
+    <row r="13" ht="22.5" customHeight="1" spans="1:9">
+      <c r="A13" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E13" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F13" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="G13" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="H13" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="I13" s="2" t="s">
+      <c r="I13" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" ht="22.5" customHeight="1">
-      <c r="A14" s="2" t="s">
+    <row r="14" ht="22.5" customHeight="1" spans="1:9">
+      <c r="A14" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="G14" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="H14" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="I14" s="2" t="s">
+      <c r="I14" s="6" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="15" ht="22.5" customHeight="1">
-      <c r="A15" s="2" t="s">
+    <row r="15" ht="22.5" customHeight="1" spans="1:9">
+      <c r="A15" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E15" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F15" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="G15" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="H15" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="I15" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="16" ht="22.5" customHeight="1">
-      <c r="A16" s="2" t="s">
+    <row r="16" ht="22.5" customHeight="1" spans="1:9">
+      <c r="A16" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="G16" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="H16" s="2" t="s">
+      <c r="H16" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="I16" s="2" t="s">
+      <c r="I16" s="6" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="17" ht="22.5" customHeight="1">
-      <c r="A17" s="2" t="s">
+    <row r="17" ht="22.5" customHeight="1" spans="1:9">
+      <c r="A17" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D17" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E17" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="F17" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="G17" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="H17" s="2" t="s">
+      <c r="H17" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="I17" s="2" t="s">
+      <c r="I17" s="6" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="18" ht="22.5" customHeight="1">
-      <c r="A18" s="2" t="s">
+    <row r="18" ht="22.5" customHeight="1" spans="1:9">
+      <c r="A18" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="E18" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="F18" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="G18" s="2" t="s">
+      <c r="G18" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="H18" s="2" t="s">
+      <c r="H18" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="I18" s="2" t="s">
+      <c r="I18" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" ht="22.5" customHeight="1">
-      <c r="A19" s="2" t="s">
+    <row r="19" ht="22.5" customHeight="1" spans="1:9">
+      <c r="A19" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D19" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="F19" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="G19" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="H19" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="I19" s="2" t="s">
+      <c r="I19" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="20" ht="22.5" customHeight="1">
-      <c r="A20" s="2" t="s">
+    <row r="20" ht="22.5" customHeight="1" spans="1:9">
+      <c r="A20" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="D20" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="E20" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="F20" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="G20" s="2" t="s">
+      <c r="G20" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="H20" s="2" t="s">
+      <c r="H20" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="I20" s="2" t="s">
+      <c r="I20" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="21" ht="22.5" customHeight="1">
-      <c r="A21" s="2" t="s">
+    <row r="21" ht="22.5" customHeight="1" spans="1:9">
+      <c r="A21" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="D21" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E21" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="F21" s="2" t="s">
+      <c r="F21" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="G21" s="2" t="s">
+      <c r="G21" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="H21" s="2" t="s">
+      <c r="H21" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="I21" s="2" t="s">
+      <c r="I21" s="6" t="s">
         <v>101</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="13.2" outlineLevelRow="5" outlineLevelCol="6"/>
+  <cols>
+    <col min="1" max="1" width="15.8888888888889" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="79.95" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2" ht="93.15" spans="1:7">
+      <c r="A2" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3" ht="93.15" spans="1:7">
+      <c r="A3" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="4" ht="119.55" spans="1:7">
+      <c r="A4" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="5" ht="132.75" spans="1:7">
+      <c r="A5" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="6" ht="93.15" spans="1:7">
+      <c r="A6" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>